<commit_message>
Adi├º├úo da 2┬¬ p├ígina do relat├│rio geral, ajustes de layout e limpeza de arquivos
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8727C2DF-832B-46CF-8B78-99DE78EAAB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D166186-A819-4FA7-8A82-74624192A7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="85">
   <si>
     <t>OS</t>
   </si>
@@ -283,6 +283,12 @@
   </si>
   <si>
     <t>APENAS DOIS OPERADORES NO DIA, FIQUEI RODANDO AS MAQUINAS COM O DIEGUINHO, MATHUES NÃO VEIO POR CAUSA DO HORARIO COMERCIAL</t>
+  </si>
+  <si>
+    <t>PROBLEMA ENCONTRADO NA MAQUINA NOVA, ROLO NO QUAL PASSA A ARTE AO CANUDO NÃO ESTÁ PEGANDO O CANUDO POR COMPLETO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SÁBADO, OPERADOR MATHUES AINDA ESTÁ NO COMERCIAL E NÃO VEM DE SÁBADO, FIQUEI AUXILIANDO NA LIMPEZA E PRODUÇÃO DO DIA </t>
   </si>
 </sst>
 </file>
@@ -2187,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S119"/>
+  <dimension ref="A1:S122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -4956,6 +4962,60 @@
         <v>66</v>
       </c>
     </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" s="2">
+        <v>46072</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D120" s="1">
+        <v>8524</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" s="2">
+        <v>46073</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D121" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="2">
+        <v>46074</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D122" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="K1:M1"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (26/02/2026  8:15:09,07)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D166186-A819-4FA7-8A82-74624192A7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B827A8-4155-4673-B16E-7963F47F9E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="85">
   <si>
     <t>OS</t>
   </si>
@@ -2193,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S122"/>
+  <dimension ref="A1:S126"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -5016,6 +5016,86 @@
         <v>17</v>
       </c>
     </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" s="2">
+        <v>46076</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D123" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124" s="2">
+        <v>46077</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D124" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" s="2">
+        <v>46078</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D125" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="2">
+        <v>46079</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D126" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G126" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="K1:M1"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (27/02/2026  8:15:08,03)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B827A8-4155-4673-B16E-7963F47F9E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3203C5D5-5D8B-4DC4-900E-A8FD24734699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="84">
   <si>
     <t>OS</t>
   </si>
@@ -286,9 +286,6 @@
   </si>
   <si>
     <t>PROBLEMA ENCONTRADO NA MAQUINA NOVA, ROLO NO QUAL PASSA A ARTE AO CANUDO NÃO ESTÁ PEGANDO O CANUDO POR COMPLETO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SÁBADO, OPERADOR MATHUES AINDA ESTÁ NO COMERCIAL E NÃO VEM DE SÁBADO, FIQUEI AUXILIANDO NA LIMPEZA E PRODUÇÃO DO DIA </t>
   </si>
 </sst>
 </file>
@@ -2193,7 +2190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S126"/>
+  <dimension ref="A1:S127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -2284,7 +2281,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>8317.5922330097092</v>
+        <v>8332.8557692307695</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -2331,12 +2328,12 @@
       <c r="I3" s="12"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>856712</v>
+        <v>866617</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>5012</v>
+        <v>5027</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -5009,8 +5006,8 @@
       <c r="F122" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G122" s="1" t="s">
-        <v>84</v>
+      <c r="G122" s="1">
+        <v>4</v>
       </c>
       <c r="H122" s="1" t="s">
         <v>17</v>
@@ -5094,6 +5091,26 @@
       </c>
       <c r="H126" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="2">
+        <v>46199</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" s="1">
+        <v>1418443</v>
+      </c>
+      <c r="D127" s="1">
+        <v>8502</v>
+      </c>
+      <c r="E127" s="1">
+        <v>9905</v>
+      </c>
+      <c r="F127" s="1">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (03/03/2026  8:15:07,32)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3203C5D5-5D8B-4DC4-900E-A8FD24734699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AE5A8E-00E1-440F-95C0-86CB6870FEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="84">
   <si>
     <t>OS</t>
   </si>
@@ -2190,7 +2190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S127"/>
+  <dimension ref="A1:S128"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -2281,7 +2281,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>8332.8557692307695</v>
+        <v>8283.5142857142855</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -2328,12 +2328,12 @@
       <c r="I3" s="12"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>866617</v>
+        <v>869769</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>5027</v>
+        <v>5087</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -5095,7 +5095,7 @@
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
-        <v>46199</v>
+        <v>46079</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>7</v>
@@ -5111,6 +5111,23 @@
       </c>
       <c r="F127" s="1">
         <v>15</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" s="2">
+        <v>46083</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D128" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E128" s="1">
+        <v>3152</v>
+      </c>
+      <c r="F128" s="1">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (05/03/2026  8:15:07,42)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AE5A8E-00E1-440F-95C0-86CB6870FEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4983C18A-9DF7-4EC6-94FA-CCF613756FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11295" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
+    <sheet name="ARTE" sheetId="2" r:id="rId2"/>
+    <sheet name="OBSERVAÇÕES" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="88">
   <si>
     <t>OS</t>
   </si>
@@ -286,6 +288,18 @@
   </si>
   <si>
     <t>PROBLEMA ENCONTRADO NA MAQUINA NOVA, ROLO NO QUAL PASSA A ARTE AO CANUDO NÃO ESTÁ PEGANDO O CANUDO POR COMPLETO</t>
+  </si>
+  <si>
+    <t>MAQUINA NOVA DE CANUDOS É REALOCADA AO SETOR DE IMPRESSÃO DIGITAL. MAQUINA VEIO, PORÉM, AINDA COM DEFEITOS E VARIAS REGULAGENS NÃO FEITAS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAQUINA AINDA EM FASE DE TESTES </t>
+  </si>
+  <si>
+    <t>OPERADOR</t>
+  </si>
+  <si>
+    <t>OBSERVAÇÃO</t>
   </si>
 </sst>
 </file>
@@ -402,7 +416,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -513,11 +527,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -600,6 +638,18 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -613,7 +663,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="54">
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -636,8 +700,122 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="18"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -792,6 +970,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1852,44 +2055,948 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>75338</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1238250</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagem 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{51F6F5F1-B4D8-48C7-AAC5-5550012616B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9447938" y="0"/>
+          <a:ext cx="1162912" cy="790575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 4" descr="SAC Plasutil| Telefones 0800 | Atendimento Online - SAC 0800">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F210745-ECF1-45B5-9C09-95741CEDF35D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="19611975" y="2981325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="AutoShape 5" descr="Crie sua loja virtual e venda sem limites! | ecomece">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91F892CF-5F2F-4483-AA06-456DEA25AE62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="19611975" y="1647825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 6" descr="Crie sua loja virtual e venda sem limites! | ecomece">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A713725-E58E-4984-AC6A-89DD84091EDD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="17802225" y="4695825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7856664-FD8F-4635-9937-C50679DFA3AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="3933825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54BA2B30-306B-4E54-AB2D-92960F25AD3B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4124325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33E80784-6187-45BC-8AAD-5BD5DDDD991E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4314825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{578B0560-EFCB-4D27-8EE0-2AAA9DCCB9F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4505325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B564022B-2E4F-4C19-A475-3824ED22DCAC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4505325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADBE6BB5-6406-486A-85D1-64DFCB7DFCD4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4695825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E30B163-772A-4A44-A90A-74EA01FE7901}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4695825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B1F6770-14D1-40F1-9C55-FCF842D56CCB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4886325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D9090B3-FCEB-4866-B26E-BFC151B28BB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="4886325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D121407-3ED3-49C4-B47D-705C9F4B7A39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="5076825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9493D31E-B7B3-4028-BF36-08C17831108E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="5076825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4189E56-E3B7-4BF0-B731-4F76C18AD2DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="5267325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64B964A9-871D-4618-A1C3-183ECCF9978A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="5267325"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="AutoShape 8" descr="Plasútil Indústria e Comércio de Plásticos Ltda | LinkedIn">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C5D3EDE-D9DC-41B4-B1F4-101C951EEBA4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15992475" y="5457825"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1296262</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21179787-183C-4A16-9737-675A8F5838B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6457950" y="0"/>
+          <a:ext cx="1162912" cy="790575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="32" dataDxfId="30" headerRowBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="29" totalsRowDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="28" totalsRowDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="27" totalsRowDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="26" totalsRowDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="25" totalsRowDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="24" totalsRowDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="23" totalsRowDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="22" totalsRowDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="42" totalsRowDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="40" totalsRowDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="38" totalsRowDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="36" totalsRowDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
   <autoFilter ref="N1:Q27" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="18" totalsRowDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24">
   <autoFilter ref="R2:S5" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
+  <autoFilter ref="A1:G1048576" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="11"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9">
+  <autoFilter ref="N1:Q27" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2190,7 +3297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA5261E-B2CC-424C-A60F-51E466D0160F}">
-  <dimension ref="A1:S128"/>
+  <dimension ref="A1:S129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="2" customWidth="1"/>
@@ -2237,11 +3344,11 @@
       <c r="J1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="28" t="s">
+      <c r="K1" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
       <c r="N1" s="15" t="s">
         <v>24</v>
       </c>
@@ -2254,10 +3361,10 @@
       <c r="Q1" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="R1" s="29" t="s">
+      <c r="R1" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="S1" s="30"/>
+      <c r="S1" s="34"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -5128,6 +6235,26 @@
       </c>
       <c r="F128" s="1">
         <v>60</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D129" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H129" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -5144,4 +6271,516 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9E4300-00AC-4831-99DB-3D8CFD1F7B78}">
+  <dimension ref="A1:Q27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="6" width="20" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" customWidth="1"/>
+    <col min="11" max="13" width="16.7109375" customWidth="1"/>
+    <col min="14" max="17" width="26.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D2" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3200</v>
+      </c>
+      <c r="F2" s="1">
+        <v>200</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="13"/>
+      <c r="J2" s="14">
+        <f>AVERAGE(E2:E206)</f>
+        <v>2600</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" s="5"/>
+      <c r="M2" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="1"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46085</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D3" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E3" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>200</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="12"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="4">
+        <f>SUM(E2:E2000)</f>
+        <v>5200</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="18">
+        <f>SUM(F2:F2000)</f>
+        <v>400</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" s="1">
+        <v>24</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>1406169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="I4" s="4">
+        <f>I2+I3</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="1">
+        <v>25</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="1">
+        <v>30</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="1">
+        <v>173</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>1353670</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="1">
+        <v>187</v>
+      </c>
+      <c r="P7" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q7" s="1"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="1">
+        <v>188</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="1"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" s="1">
+        <v>190</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q9" s="1"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" s="1">
+        <v>411</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" s="1">
+        <v>474</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q11" s="1"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="1">
+        <v>475</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q12" s="1"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="1">
+        <v>476</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" s="1"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="1">
+        <v>477</v>
+      </c>
+      <c r="P14" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>1389060</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="1">
+        <v>596</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q15" s="1"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="N16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O16" s="1">
+        <v>639</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q16" s="1"/>
+    </row>
+    <row r="17" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O17" s="1">
+        <v>647</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q17" s="1"/>
+    </row>
+    <row r="18" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" s="1">
+        <v>648</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q18" s="1"/>
+    </row>
+    <row r="19" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O19" s="1">
+        <v>649</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q19" s="1"/>
+    </row>
+    <row r="20" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N20" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O20" s="1">
+        <v>767</v>
+      </c>
+      <c r="P20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q20" s="1"/>
+    </row>
+    <row r="21" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O21" s="1">
+        <v>888</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q21" s="1"/>
+    </row>
+    <row r="22" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N22" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1149</v>
+      </c>
+      <c r="P22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>1404598</v>
+      </c>
+    </row>
+    <row r="23" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1157</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q23" s="1"/>
+    </row>
+    <row r="24" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N24" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O24" s="1">
+        <v>1174</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>308564</v>
+      </c>
+    </row>
+    <row r="25" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O25" s="1">
+        <v>1202</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O26" s="1">
+        <v>1345</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="14:17" x14ac:dyDescent="0.25">
+      <c r="N27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O27" s="1">
+        <v>1498</v>
+      </c>
+      <c r="P27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q27" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="K1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B5184B-1E33-47EF-9675-0892F220B5E2}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="23.7109375" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (06/03/2026  8:15:07,95)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4983C18A-9DF7-4EC6-94FA-CCF613756FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259A7AE-31C0-45C7-99B6-54B94C158276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="90">
   <si>
     <t>OS</t>
   </si>
@@ -300,6 +300,12 @@
   </si>
   <si>
     <t>OBSERVAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAQUINA APRESENTA DEFEITO NO ROLO QUE PASSA AS ARTES PARA O CANUDO, ROLO RACHOU POR COMPLETO </t>
+  </si>
+  <si>
+    <t>05/03/20206</t>
   </si>
 </sst>
 </file>
@@ -663,7 +669,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="60">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <border outline="0">
         <top style="thin">
@@ -2866,13 +2890,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1296262</xdr:colOff>
+      <xdr:colOff>1277212</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
@@ -2903,7 +2927,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6457950" y="0"/>
+          <a:off x="6438900" y="0"/>
           <a:ext cx="1162912" cy="790575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2917,84 +2941,84 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}" name="Tabela5" displayName="Tabela5" ref="A1:H1048576" totalsRowCount="1" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58">
   <autoFilter ref="A1:H1048575" xr:uid="{5BB2D3F9-C887-4B4C-B99D-D2DF65DEC2A6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="36" totalsRowDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{087A0113-3A7F-4ED4-85E5-B6DA7A785E6E}" name="Data" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{B5ACDCB9-111C-4EEF-A7F2-0DFD4B46F701}" name="Turno" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{8DF57E4B-CE5D-4D81-A024-AF995D46B0D6}" name="OS" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{ED2D14F5-1612-4387-8474-BB902D6983C6}" name="Operador" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{98386C95-9775-4F1F-A3CC-9A16E030AF66}" name="Produzidos" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{3F049097-8486-4DDD-93F7-CCC691CC4860}" name="Perdas" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{26B92E51-FF95-433C-9069-C56C7828476A}" name="Observação" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{8B43B335-323F-4C61-82F4-07648230810B}" name="Coluna1" dataDxfId="42" totalsRowDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}" name="Tabela1" displayName="Tabela1" ref="N1:Q27" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39">
   <autoFilter ref="N1:Q27" xr:uid="{89285ECA-F282-4F01-A009-CC89A51CDC7A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{EDE6611D-5889-4C5E-8516-947DDEFF7DCC}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{7D1A3E97-C617-4FD2-B05B-A97B6AD5F90C}" name="CORES" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{03E79F60-8E38-46EF-92B4-918A623037DE}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{1B33BBDF-2D4E-45C0-873F-D04B114DCBBF}" name="os" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}" name="Tabela4" displayName="Tabela4" ref="R2:S5" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30">
   <autoFilter ref="R2:S5" xr:uid="{1FE77D6E-600C-406D-AA64-535CF7AD02D9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{065934BB-F4F9-47CC-8C25-186E2F5FD276}" name="NOME" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{5F9476BD-3CB7-480B-BA25-725A0FDEB9A9}" name="RAMAL" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}" name="Tabela3" displayName="Tabela3" ref="A1:G1048576" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
   <autoFilter ref="A1:G1048576" xr:uid="{CA95B68F-F434-4033-BFD9-2BB1AA7C7BF7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{0280B923-DB87-4E28-A2B5-2ABF26E67A3C}" name="Data" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{CDEDA308-953F-46E8-8272-8EB68D248564}" name="Turno" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{A09724A8-B36D-4AD5-98B7-ADD526A91EFB}" name="OS" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{AF64C0A2-C8AC-47A7-BF73-70D43293AAAA}" name="Operador" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{F74EB60A-3874-4909-8B14-62AD3728B999}" name="Produzidos" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{124854EA-F6BE-4A3F-B8F0-8D4078EF15EC}" name="Perdas" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{FAD2623B-15B5-49D0-88AC-906319948EA0}" name="Observação" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}" name="Tabela17" displayName="Tabela17" ref="N1:Q27" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15">
   <autoFilter ref="N1:Q27" xr:uid="{7C61B123-99B4-407D-925F-D62D7C54D232}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E76169FA-FCD1-44CA-96FF-791C61B530A3}" name="CANUDOS " totalsRowLabel="Total" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{35FFF8DF-05B8-44FE-B351-F847EE90084A}" name="CORES" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9A289D66-8372-477D-979D-D9E4A4CA121C}" name="DESCRIÇÃO" totalsRowFunction="count" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0D9D8711-FBB3-4387-B4D2-D3D4718A6B6D}" name="os" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" headerRowBorderDxfId="1" tableBorderDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="6">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6434,6 +6458,24 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46086</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1">
+        <v>8524</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" t="s">
+        <v>17</v>
+      </c>
       <c r="I4" s="4">
         <f>I2+I3</f>
         <v>0</v>
@@ -6752,11 +6794,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6B5184B-1E33-47EF-9675-0892F220B5E2}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="23.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="1" max="4" width="23.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -6774,6 +6816,23 @@
       </c>
       <c r="E1" s="31" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
+        <v>8524</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica (07/03/2026  8:15:07,56)
</commit_message>
<xml_diff>
--- a/Canudos.xlsx
+++ b/Canudos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2259A7AE-31C0-45C7-99B6-54B94C158276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766FECA2-ED9B-495E-898D-877A07362EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2551C110-448D-4C8A-AC10-E46F4B669B16}"/>
   </bookViews>
   <sheets>
     <sheet name="ENCABEÇAMENTO" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="91">
   <si>
     <t>OS</t>
   </si>
@@ -306,6 +306,9 @@
   </si>
   <si>
     <t>05/03/20206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VOLTA DA MAQUINA 29, OPERADOR AUXILIOU NAS MAQUINAS DE IMPRESSÃO ENQUANTO OPERADOR DIEGO FAZIA TESTES E DPS TROCAVA MOLDE PARA NOVA ORDEM </t>
   </si>
 </sst>
 </file>
@@ -686,14 +689,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -3011,14 +3014,14 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}" name="Tabela7" displayName="Tabela7" ref="A1:E1048576" totalsRowShown="0" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
   <autoFilter ref="A1:E1048576" xr:uid="{B6F26BC4-2F5B-4DD0-B255-2DBF5E945A60}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{A457A19A-4874-4397-B513-B6F9A3B0A60A}" name="Data" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{95C69B8D-1A39-40CB-B5FA-F58DC3500DA7}" name="Turno" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{046BEC21-BC63-4C71-8608-9399078C3481}" name="OPERADOR" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{C3B0A1FD-B664-4E6E-9624-C807349AADDB}" name="OBSERVAÇÃO" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C7967862-84A2-4EDD-9459-5C2DFCE69540}" name="Coluna1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6388,7 +6391,7 @@
       <c r="I2" s="13"/>
       <c r="J2" s="14">
         <f>AVERAGE(E2:E206)</f>
-        <v>2600</v>
+        <v>1854.6666666666667</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>13</v>
@@ -6437,12 +6440,12 @@
       <c r="J3" s="1"/>
       <c r="K3" s="4">
         <f>SUM(E2:E2000)</f>
-        <v>5200</v>
+        <v>5564</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="18">
         <f>SUM(F2:F2000)</f>
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>27</v>
@@ -6496,6 +6499,30 @@
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>46087</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1406169</v>
+      </c>
+      <c r="D5" s="1">
+        <v>8524</v>
+      </c>
+      <c r="E5" s="1">
+        <v>364</v>
+      </c>
+      <c r="F5" s="1">
+        <v>100</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" t="s">
+        <v>17</v>
+      </c>
       <c r="N5" s="1" t="s">
         <v>27</v>
       </c>

</xml_diff>